<commit_message>
Bulk-migrate all adventure detail pages
Add the remaining 15 adventure child pages to the adventures URL list and import
them through the existing adventures template — reusing breadcrumb, carousel
(hero-img), columns (spec), and tabs (adventure) with the yellow-underline title
and adventure-body layout, consistent with bali-surf-camp.

16 pages imported (92–98% completeness), 0 failures.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventures.report.xlsx
+++ b/tools/importer/reports/import-adventures.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="98">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,13 +73,238 @@
     <t>adventures</t>
   </si>
   <si>
-    <t>2026-09-14T08:37:48.508Z</t>
+    <t>2026-09-14T09:44:15.765Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:44:20.894Z</t>
+  </si>
+  <si>
+    <t>Beervana in Portland</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:44:27.506Z</t>
+  </si>
+  <si>
+    <t>Climbing New Zealand</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:44:32.133Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:44:37.121Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:44:43.436Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:44:49.182Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:44:54.071Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:45:00.294Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:45:05.831Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:45:10.545Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:45:14.883Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:45:20.379Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:45:26.716Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:45:30.892Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-14T09:45:36.457Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
   </si>
 </sst>
 </file>
@@ -468,12 +693,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="33" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
@@ -558,6 +782,396 @@
         <v>22</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" t="s">
+        <v>65</v>
+      </c>
+      <c r="G12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" t="s">
+        <v>71</v>
+      </c>
+      <c r="H13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" t="s">
+        <v>75</v>
+      </c>
+      <c r="G14" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" t="s">
+        <v>85</v>
+      </c>
+      <c r="G16" t="s">
+        <v>86</v>
+      </c>
+      <c r="H16" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" t="s">
+        <v>91</v>
+      </c>
+      <c r="H17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" t="s">
+        <v>96</v>
+      </c>
+      <c r="H18" t="s">
+        <v>97</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix adventure-list filter hiding and stray activity metadata block
- adventure-list: filtered-out cards stayed visible because the
  `.adventure-card { display: flex }` class selector outranks the [hidden]
  attribute's default `display: none`. Add an explicit
  `.adventure-card[hidden] { display: none }` rule so activity filtering
  actually hides non-matching cards.
- import-adventures: the activity tag was emitted as a SECOND Metadata block,
  which EDS does not merge — it rendered as a visible "activity / <value>"
  block on every adventure detail page. Merge the activity row into the single
  metadata block createMetadata produces instead, so it becomes an invisible
  <meta name="activity"> head tag while still driving the dynamic listing.
  Re-imported all 16 adventure pages (reports updated).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventures.report.xlsx
+++ b/tools/importer/reports/import-adventures.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="182">
   <si>
     <t>_reportFile</t>
   </si>
@@ -70,7 +70,136 @@
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["cards-people","cards-people","cards-people","cards-people","cards-people","cards-people","cards-people"]</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>about-us</t>
+  </si>
+  <si>
+    <t>2026-09-14T18:16:29.575Z</t>
+  </si>
+  <si>
+    <t>About Us</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures.report.json</t>
+  </si>
+  <si>
+    <t>["carousel","adventure-list","adventure-list","adventure-list","adventure-list","adventure-list","adventure-list"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures</t>
+  </si>
+  <si>
+    <t>adventures-landing</t>
+  </si>
+  <si>
+    <t>2026-09-14T11:48:04.413Z</t>
+  </si>
+  <si>
+    <t>Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures.html</t>
+  </si>
+  <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>["accordion"]</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>faqs</t>
+  </si>
+  <si>
+    <t>2026-09-14T15:15:52.540Z</t>
+  </si>
+  <si>
+    <t>FAQs</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine.report.json</t>
+  </si>
+  <si>
+    <t>["columns","cards","cards-secure","cards-secure"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine</t>
+  </si>
+  <si>
+    <t>magazine</t>
+  </si>
+  <si>
+    <t>2026-09-14T12:11:58.324Z</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
     <t>us/en/adventures/bali-surf-camp.html.report.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: metaBlock.querySelector is not a function
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: metaBlock.querySelector is not a function
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30
+    at processUrl (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:691:31)
+    at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:954:22)</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-09-14T18:41:29.034Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb","carousel","columns","tabs"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventures</t>
+  </si>
+  <si>
+    <t>2026-09-14T18:42:15.840Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.html.report.json</t>
   </si>
   <si>
     <t xml:space="preserve">page.evaluate: Error: Failed to import page: metaBlock.append is not a function
@@ -85,39 +214,6 @@
     at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:954:22)</t>
   </si>
   <si>
-    <t>us/en/adventures/bali-surf-camp.html</t>
-  </si>
-  <si>
-    <t>failed</t>
-  </si>
-  <si>
-    <t>2026-09-14T10:59:31.819Z</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/bali-surf-camp.report.json</t>
-  </si>
-  <si>
-    <t>["breadcrumb","carousel","columns","tabs"]</t>
-  </si>
-  <si>
-    <t>us/en/adventures/bali-surf-camp</t>
-  </si>
-  <si>
-    <t>adventures</t>
-  </si>
-  <si>
-    <t>2026-09-14T11:00:09.445Z</t>
-  </si>
-  <si>
-    <t>Bali Surf Camp</t>
-  </si>
-  <si>
-    <t>us/en/adventures/beervana-portland.html.report.json</t>
-  </si>
-  <si>
     <t>us/en/adventures/beervana-portland.html</t>
   </si>
   <si>
@@ -133,7 +229,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:15.307Z</t>
+    <t>2026-09-14T18:42:20.466Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -157,7 +253,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:20.206Z</t>
+    <t>2026-09-14T18:42:26.387Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -181,7 +277,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:24.848Z</t>
+    <t>2026-09-14T18:42:31.422Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -205,7 +301,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:31.131Z</t>
+    <t>2026-09-14T18:42:37.023Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -229,7 +325,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:34.811Z</t>
+    <t>2026-09-14T18:42:42.948Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -253,7 +349,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:39.962Z</t>
+    <t>2026-09-14T18:42:47.711Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -277,7 +373,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:43.916Z</t>
+    <t>2026-09-14T18:42:53.912Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -301,7 +397,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:50.670Z</t>
+    <t>2026-09-14T18:42:58.918Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -325,7 +421,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:55.192Z</t>
+    <t>2026-09-14T18:43:04.684Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -349,7 +445,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:59.840Z</t>
+    <t>2026-09-14T18:43:10.461Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -373,7 +469,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:04.096Z</t>
+    <t>2026-09-14T18:43:15.201Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -397,7 +493,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:07.840Z</t>
+    <t>2026-09-14T18:43:19.845Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -421,7 +517,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:12.189Z</t>
+    <t>2026-09-14T18:43:23.793Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -445,7 +541,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:17.884Z</t>
+    <t>2026-09-14T18:43:29.226Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -469,7 +565,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:22.539Z</t>
+    <t>2026-09-14T18:43:34.744Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -861,11 +957,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="26" customWidth="1"/>
     <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="50" customWidth="1"/>
@@ -940,28 +1036,28 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
         <v>22</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>23</v>
       </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>24</v>
-      </c>
-      <c r="I3" t="s">
-        <v>12</v>
       </c>
       <c r="J3" t="s">
         <v>25</v>
@@ -996,47 +1092,47 @@
         <v>31</v>
       </c>
       <c r="J4" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I5" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="J5" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -1045,62 +1141,62 @@
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F6" t="s">
         <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="I6" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="J6" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G7" t="s">
         <v>12</v>
       </c>
       <c r="H7" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="I7" t="s">
         <v>12</v>
       </c>
       <c r="J7" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
@@ -1109,62 +1205,62 @@
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="F8" t="s">
         <v>14</v>
       </c>
       <c r="G8" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H8" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="I8" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="J8" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G9" t="s">
         <v>12</v>
       </c>
       <c r="H9" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
         <v>12</v>
       </c>
       <c r="J9" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1173,62 +1269,62 @@
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="F10" t="s">
         <v>14</v>
       </c>
       <c r="G10" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H10" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G11" t="s">
         <v>12</v>
       </c>
       <c r="H11" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="I11" t="s">
         <v>12</v>
       </c>
       <c r="J11" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
@@ -1237,62 +1333,62 @@
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="F12" t="s">
         <v>14</v>
       </c>
       <c r="G12" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="J12" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E13" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G13" t="s">
         <v>12</v>
       </c>
       <c r="H13" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="I13" t="s">
         <v>12</v>
       </c>
       <c r="J13" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -1301,62 +1397,62 @@
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="I14" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="J14" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E15" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G15" t="s">
         <v>12</v>
       </c>
       <c r="H15" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="I15" t="s">
         <v>12</v>
       </c>
       <c r="J15" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C16" t="s">
         <v>12</v>
@@ -1365,62 +1461,62 @@
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="F16" t="s">
         <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H16" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="I16" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="J16" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="F17" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G17" t="s">
         <v>12</v>
       </c>
       <c r="H17" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="I17" t="s">
         <v>12</v>
       </c>
       <c r="J17" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
         <v>12</v>
@@ -1429,62 +1525,62 @@
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H18" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="I18" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="J18" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
       </c>
       <c r="C19" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E19" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="F19" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G19" t="s">
         <v>12</v>
       </c>
       <c r="H19" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="I19" t="s">
         <v>12</v>
       </c>
       <c r="J19" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -1493,62 +1589,62 @@
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H20" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="I20" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="J20" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D21" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E21" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="F21" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G21" t="s">
         <v>12</v>
       </c>
       <c r="H21" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="I21" t="s">
         <v>12</v>
       </c>
       <c r="J21" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="B22" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -1557,62 +1653,62 @@
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H22" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="I22" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="J22" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="B23" t="s">
         <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E23" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="F23" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G23" t="s">
         <v>12</v>
       </c>
       <c r="H23" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="I23" t="s">
         <v>12</v>
       </c>
       <c r="J23" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="B24" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -1621,62 +1717,62 @@
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="F24" t="s">
         <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H24" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="I24" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="J24" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B25" t="s">
         <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E25" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="F25" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G25" t="s">
         <v>12</v>
       </c>
       <c r="H25" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="I25" t="s">
         <v>12</v>
       </c>
       <c r="J25" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="B26" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -1685,62 +1781,62 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H26" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="I26" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="J26" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E27" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="F27" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G27" t="s">
         <v>12</v>
       </c>
       <c r="H27" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="I27" t="s">
         <v>12</v>
       </c>
       <c r="J27" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="B28" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C28" t="s">
         <v>12</v>
@@ -1749,62 +1845,62 @@
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="F28" t="s">
         <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H28" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="I28" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="J28" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B29" t="s">
         <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E29" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="F29" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G29" t="s">
         <v>12</v>
       </c>
       <c r="H29" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="I29" t="s">
         <v>12</v>
       </c>
       <c r="J29" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B30" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
@@ -1813,62 +1909,62 @@
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="F30" t="s">
         <v>14</v>
       </c>
       <c r="G30" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H30" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="I30" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="J30" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B31" t="s">
         <v>12</v>
       </c>
       <c r="C31" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E31" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="F31" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G31" t="s">
         <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="I31" t="s">
         <v>12</v>
       </c>
       <c r="J31" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="B32" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -1877,62 +1973,62 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H32" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="I32" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="J32" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="B33" t="s">
         <v>12</v>
       </c>
       <c r="C33" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="D33" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="E33" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="F33" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G33" t="s">
         <v>12</v>
       </c>
       <c r="H33" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="I33" t="s">
         <v>12</v>
       </c>
       <c r="J33" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="B34" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
@@ -1941,22 +2037,150 @@
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="H34" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="I34" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="J34" t="s">
-        <v>147</v>
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>166</v>
+      </c>
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" t="s">
+        <v>61</v>
+      </c>
+      <c r="D35" t="s">
+        <v>62</v>
+      </c>
+      <c r="E35" t="s">
+        <v>167</v>
+      </c>
+      <c r="F35" t="s">
+        <v>51</v>
+      </c>
+      <c r="G35" t="s">
+        <v>12</v>
+      </c>
+      <c r="H35" t="s">
+        <v>168</v>
+      </c>
+      <c r="I35" t="s">
+        <v>12</v>
+      </c>
+      <c r="J35" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>170</v>
+      </c>
+      <c r="B36" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
+        <v>171</v>
+      </c>
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>57</v>
+      </c>
+      <c r="H36" t="s">
+        <v>172</v>
+      </c>
+      <c r="I36" t="s">
+        <v>173</v>
+      </c>
+      <c r="J36" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>174</v>
+      </c>
+      <c r="B37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" t="s">
+        <v>61</v>
+      </c>
+      <c r="D37" t="s">
+        <v>62</v>
+      </c>
+      <c r="E37" t="s">
+        <v>175</v>
+      </c>
+      <c r="F37" t="s">
+        <v>51</v>
+      </c>
+      <c r="G37" t="s">
+        <v>12</v>
+      </c>
+      <c r="H37" t="s">
+        <v>176</v>
+      </c>
+      <c r="I37" t="s">
+        <v>12</v>
+      </c>
+      <c r="J37" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>178</v>
+      </c>
+      <c r="B38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" t="s">
+        <v>179</v>
+      </c>
+      <c r="F38" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>57</v>
+      </c>
+      <c r="H38" t="s">
+        <v>180</v>
+      </c>
+      <c r="I38" t="s">
+        <v>181</v>
+      </c>
+      <c r="J38" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>